<commit_message>
İş Takip Güncellemesi - 16.09.2026 16:20:55
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -4033,7 +4033,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L95" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="96">
@@ -4071,7 +4071,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L96" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="97">
@@ -4192,7 +4192,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L99" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="100" xml:space="preserve">
@@ -4230,7 +4230,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L100" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
       <c r="M100" t="str" xml:space="preserve">
         <v xml:space="preserve">15.10.2025 Projesine başlanılacak(Ormancı kontrolünde)_x000d__x000d__x000d_
@@ -4320,7 +4320,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L102" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
       <c r="M102" t="str" xml:space="preserve">
         <v xml:space="preserve">01.11.2025 firmaya teslim edilecek_x000d__x000d_
@@ -4412,7 +4412,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L104" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="105">
@@ -4450,7 +4450,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L105" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
       <c r="M105" t="str">
         <v>[x] 21.10.2025 komisyon yapılacak(İsmail Pehlivan)</v>
@@ -4491,7 +4491,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L106" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
       <c r="M106" t="str" xml:space="preserve">
         <v xml:space="preserve">03.11.2025 firmaya teslim edilecek_x000d__x000d_
@@ -4542,7 +4542,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L107" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
       <c r="M107" t="str" xml:space="preserve">
         <v xml:space="preserve">16.10.2025 firmaya teslim edilecek_x000d__x000d__x000d_
@@ -4668,7 +4668,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L110" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
       <c r="M110" t="str" xml:space="preserve">
         <v xml:space="preserve">16.10.2025 Taşçılı tutanak Kadastro Üyesine teslim edilecek._x000d__x000d__x000d_
@@ -4716,7 +4716,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L111" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
       <c r="M111" t="str" xml:space="preserve">
         <v xml:space="preserve">24.10.2025 firmaya teslim edilecek_x000d__x000d_
@@ -4767,7 +4767,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L112" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
       <c r="M112" t="str">
         <v>[x] 20.10.2025 askıya çıkacak</v>
@@ -4854,7 +4854,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L114" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
       <c r="M114" t="str" xml:space="preserve">
         <v xml:space="preserve">14.11.2025 firmaya teslim edilecek_x000d__x000d_
@@ -4902,7 +4902,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L115" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
       <c r="M115" t="str" xml:space="preserve">
         <v xml:space="preserve">Kıymetlendirmede eksiklikler var firma tamamlayacak bu hafta(20.10.2025)_x000d__x000d_
@@ -5001,7 +5001,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L117" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
       <c r="M117" t="str" xml:space="preserve">
         <v xml:space="preserve">01.11.2025 firmaya teslim edilecek_x000d__x000d__x000d_
@@ -5052,7 +5052,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L118" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
       <c r="M118" t="str" xml:space="preserve">
         <v xml:space="preserve">01.11.2025 firmaya teslim edilecek_x000d__x000d_
@@ -5195,7 +5195,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L121" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
       <c r="M121" t="str" xml:space="preserve">
         <v xml:space="preserve">17.10.2025 firmaya teslim edilecek_x000d__x000d__x000d_
@@ -5244,7 +5244,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L122" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
       <c r="M122" t="str" xml:space="preserve">
         <v xml:space="preserve">17.10.2025 Tutanaklara başlanılacak_x000d__x000d__x000d_

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 06.10.2026 11:08:57
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -7462,7 +7462,7 @@
         <v/>
       </c>
       <c r="L180" t="str">
-        <v>VERİLER ELEKTRONİK ORTAMDA HAZIRLANDI.</v>
+        <v>DEĞERLENDİRMEDE</v>
       </c>
     </row>
     <row r="181">
@@ -7771,7 +7771,7 @@
     </row>
     <row r="189">
       <c r="A189" t="str">
-        <v>HAYIR</v>
+        <v>EVET</v>
       </c>
       <c r="B189" t="str">
         <v>Mut</v>
@@ -7809,7 +7809,7 @@
     </row>
     <row r="190">
       <c r="A190" t="str">
-        <v>HAYIR</v>
+        <v>EVET</v>
       </c>
       <c r="B190" t="str">
         <v>Mut</v>
@@ -7880,7 +7880,7 @@
         <v/>
       </c>
       <c r="L191" t="str">
-        <v>ASKI İLANINA HAZIRLANIYOR</v>
+        <v>KESİN ASKIDA</v>
       </c>
     </row>
     <row r="192">
@@ -8236,7 +8236,7 @@
     </row>
     <row r="201" xml:space="preserve">
       <c r="A201" t="str">
-        <v>HAYIR</v>
+        <v>EVET</v>
       </c>
       <c r="B201" t="str">
         <v>Gülnar</v>

</xml_diff>